<commit_message>
Start Phase 3, Revise schedule template
</commit_message>
<xml_diff>
--- a/DATA/schedule.xlsx
+++ b/DATA/schedule.xlsx
@@ -11,15 +11,14 @@
     <sheet name="Tuesday" sheetId="2" r:id="rId2"/>
     <sheet name="Wednesday" sheetId="3" r:id="rId3"/>
     <sheet name="Thursday" sheetId="4" r:id="rId4"/>
-    <sheet name="Sunday" sheetId="5" r:id="rId5"/>
-    <sheet name="All Assignments" sheetId="6" r:id="rId6"/>
+    <sheet name="All Assignments" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="46">
   <si>
     <t>Monday - [Insert Date]</t>
   </si>
@@ -51,34 +50,58 @@
     <t>Comments / Late</t>
   </si>
   <si>
-    <t>Ref1</t>
-  </si>
-  <si>
-    <t>TBD</t>
-  </si>
-  <si>
-    <t>Ref2</t>
+    <t>Chisholm Teddy</t>
+  </si>
+  <si>
+    <t>Court 1</t>
+  </si>
+  <si>
+    <t>Court 2</t>
+  </si>
+  <si>
+    <t>Enkhjargal Manlai</t>
   </si>
   <si>
     <t>-</t>
   </si>
   <si>
-    <t>Ref3</t>
-  </si>
-  <si>
-    <t>Ref4</t>
-  </si>
-  <si>
-    <t>Ref5</t>
-  </si>
-  <si>
-    <t>Ref6</t>
-  </si>
-  <si>
-    <t>Ref7</t>
-  </si>
-  <si>
-    <t>Ref8</t>
+    <t>Court 3</t>
+  </si>
+  <si>
+    <t>Gray Caroline</t>
+  </si>
+  <si>
+    <t>Huang Jason</t>
+  </si>
+  <si>
+    <t>Kerrigan Declan</t>
+  </si>
+  <si>
+    <t>Kevin Huang</t>
+  </si>
+  <si>
+    <t>Little Patrick</t>
+  </si>
+  <si>
+    <t>Nguyen Jinnie</t>
+  </si>
+  <si>
+    <t>Nguyen Millie</t>
+  </si>
+  <si>
+    <t>Pineo Kyle</t>
+  </si>
+  <si>
+    <t>Roix Aiden</t>
+  </si>
+  <si>
+    <t>Wasser David</t>
+  </si>
+  <si>
+    <t>Xu Ryan</t>
+  </si>
+  <si>
+    <t>Zaya Maria</t>
   </si>
   <si>
     <t>Tuesday - [Insert Date]</t>
@@ -90,9 +113,6 @@
     <t>Thursday - [Insert Date]</t>
   </si>
   <si>
-    <t>Sunday - [Insert Date]</t>
-  </si>
-  <si>
     <t>All Assignments - [Insert Date]</t>
   </si>
   <si>
@@ -108,37 +128,34 @@
     <t>Thursday</t>
   </si>
   <si>
-    <t>Sunday</t>
-  </si>
-  <si>
     <t>6:30, 7:30, 8:30, 9:30, 10:30</t>
   </si>
   <si>
+    <t>7:30, 8:30, 9:30, 10:30</t>
+  </si>
+  <si>
     <t>6:30, 7:30, 8:30</t>
   </si>
   <si>
+    <t>6:30, 7:30, 8:30, 9:30</t>
+  </si>
+  <si>
+    <t>8:30, 9:30, 10:30</t>
+  </si>
+  <si>
+    <t>6:30, 8:30</t>
+  </si>
+  <si>
     <t>9:30, 10:30</t>
   </si>
   <si>
-    <t>7:30, 8:30</t>
-  </si>
-  <si>
-    <t>7:30, 8:30, 9:30</t>
-  </si>
-  <si>
     <t>8:30, 9:30</t>
   </si>
   <si>
+    <t>6:30, 8:30, 9:30, 10:30</t>
+  </si>
+  <si>
     <t>6:30, 7:30</t>
-  </si>
-  <si>
-    <t>6:30, 7:30, 8:30, 10:30</t>
-  </si>
-  <si>
-    <t>7:30, 8:30, 9:30, 10:30</t>
-  </si>
-  <si>
-    <t>6:30, 7:30, 8:30, 9:30</t>
   </si>
 </sst>
 </file>
@@ -536,7 +553,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z11"/>
+  <dimension ref="A1:Z17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" customWidth="1"/>
@@ -636,7 +653,7 @@
         <v>11</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>11</v>
@@ -650,22 +667,22 @@
     </row>
     <row r="5" spans="1:26">
       <c r="A5" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -676,22 +693,22 @@
     </row>
     <row r="6" spans="1:26">
       <c r="A6" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -702,22 +719,22 @@
     </row>
     <row r="7" spans="1:26">
       <c r="A7" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -728,22 +745,22 @@
     </row>
     <row r="8" spans="1:26">
       <c r="A8" s="2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -754,22 +771,22 @@
     </row>
     <row r="9" spans="1:26">
       <c r="A9" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -780,19 +797,19 @@
     </row>
     <row r="10" spans="1:26">
       <c r="A10" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>11</v>
@@ -806,22 +823,22 @@
     </row>
     <row r="11" spans="1:26">
       <c r="A11" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -829,6 +846,162 @@
       <c r="J11" s="4"/>
       <c r="K11" s="4"/>
       <c r="L11" s="3"/>
+    </row>
+    <row r="12" spans="1:26">
+      <c r="A12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G12" s="4"/>
+      <c r="H12" s="4"/>
+      <c r="I12" s="4"/>
+      <c r="J12" s="4"/>
+      <c r="K12" s="4"/>
+      <c r="L12" s="3"/>
+    </row>
+    <row r="13" spans="1:26">
+      <c r="A13" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
+      <c r="I13" s="4"/>
+      <c r="J13" s="4"/>
+      <c r="K13" s="4"/>
+      <c r="L13" s="3"/>
+    </row>
+    <row r="14" spans="1:26">
+      <c r="A14" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G14" s="4"/>
+      <c r="H14" s="4"/>
+      <c r="I14" s="4"/>
+      <c r="J14" s="4"/>
+      <c r="K14" s="4"/>
+      <c r="L14" s="3"/>
+    </row>
+    <row r="15" spans="1:26">
+      <c r="A15" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G15" s="4"/>
+      <c r="H15" s="4"/>
+      <c r="I15" s="4"/>
+      <c r="J15" s="4"/>
+      <c r="K15" s="4"/>
+      <c r="L15" s="3"/>
+    </row>
+    <row r="16" spans="1:26">
+      <c r="A16" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G16" s="4"/>
+      <c r="H16" s="4"/>
+      <c r="I16" s="4"/>
+      <c r="J16" s="4"/>
+      <c r="K16" s="4"/>
+      <c r="L16" s="3"/>
+    </row>
+    <row r="17" spans="1:12">
+      <c r="A17" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G17" s="4"/>
+      <c r="H17" s="4"/>
+      <c r="I17" s="4"/>
+      <c r="J17" s="4"/>
+      <c r="K17" s="4"/>
+      <c r="L17" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -842,7 +1015,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z11"/>
+  <dimension ref="A1:Z17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" customWidth="1"/>
@@ -852,7 +1025,7 @@
   <sheetData>
     <row r="1" spans="1:26" ht="25" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -933,19 +1106,19 @@
         <v>10</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>11</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -956,22 +1129,22 @@
     </row>
     <row r="5" spans="1:26">
       <c r="A5" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -982,22 +1155,22 @@
     </row>
     <row r="6" spans="1:26">
       <c r="A6" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>11</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -1008,22 +1181,22 @@
     </row>
     <row r="7" spans="1:26">
       <c r="A7" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -1034,22 +1207,22 @@
     </row>
     <row r="8" spans="1:26">
       <c r="A8" s="2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -1060,22 +1233,22 @@
     </row>
     <row r="9" spans="1:26">
       <c r="A9" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -1086,22 +1259,22 @@
     </row>
     <row r="10" spans="1:26">
       <c r="A10" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -1112,22 +1285,22 @@
     </row>
     <row r="11" spans="1:26">
       <c r="A11" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -1135,6 +1308,162 @@
       <c r="J11" s="4"/>
       <c r="K11" s="4"/>
       <c r="L11" s="3"/>
+    </row>
+    <row r="12" spans="1:26">
+      <c r="A12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" s="4"/>
+      <c r="H12" s="4"/>
+      <c r="I12" s="4"/>
+      <c r="J12" s="4"/>
+      <c r="K12" s="4"/>
+      <c r="L12" s="3"/>
+    </row>
+    <row r="13" spans="1:26">
+      <c r="A13" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
+      <c r="I13" s="4"/>
+      <c r="J13" s="4"/>
+      <c r="K13" s="4"/>
+      <c r="L13" s="3"/>
+    </row>
+    <row r="14" spans="1:26">
+      <c r="A14" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G14" s="4"/>
+      <c r="H14" s="4"/>
+      <c r="I14" s="4"/>
+      <c r="J14" s="4"/>
+      <c r="K14" s="4"/>
+      <c r="L14" s="3"/>
+    </row>
+    <row r="15" spans="1:26">
+      <c r="A15" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G15" s="4"/>
+      <c r="H15" s="4"/>
+      <c r="I15" s="4"/>
+      <c r="J15" s="4"/>
+      <c r="K15" s="4"/>
+      <c r="L15" s="3"/>
+    </row>
+    <row r="16" spans="1:26">
+      <c r="A16" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G16" s="4"/>
+      <c r="H16" s="4"/>
+      <c r="I16" s="4"/>
+      <c r="J16" s="4"/>
+      <c r="K16" s="4"/>
+      <c r="L16" s="3"/>
+    </row>
+    <row r="17" spans="1:12">
+      <c r="A17" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G17" s="4"/>
+      <c r="H17" s="4"/>
+      <c r="I17" s="4"/>
+      <c r="J17" s="4"/>
+      <c r="K17" s="4"/>
+      <c r="L17" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1148,7 +1477,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z11"/>
+  <dimension ref="A1:Z17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" customWidth="1"/>
@@ -1158,7 +1487,7 @@
   <sheetData>
     <row r="1" spans="1:26" ht="25" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1239,19 +1568,19 @@
         <v>10</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -1262,22 +1591,22 @@
     </row>
     <row r="5" spans="1:26">
       <c r="A5" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -1288,22 +1617,22 @@
     </row>
     <row r="6" spans="1:26">
       <c r="A6" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -1314,22 +1643,22 @@
     </row>
     <row r="7" spans="1:26">
       <c r="A7" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -1340,22 +1669,22 @@
     </row>
     <row r="8" spans="1:26">
       <c r="A8" s="2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -1366,22 +1695,22 @@
     </row>
     <row r="9" spans="1:26">
       <c r="A9" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -1392,22 +1721,22 @@
     </row>
     <row r="10" spans="1:26">
       <c r="A10" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -1418,22 +1747,22 @@
     </row>
     <row r="11" spans="1:26">
       <c r="A11" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -1441,6 +1770,162 @@
       <c r="J11" s="4"/>
       <c r="K11" s="4"/>
       <c r="L11" s="3"/>
+    </row>
+    <row r="12" spans="1:26">
+      <c r="A12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" s="4"/>
+      <c r="H12" s="4"/>
+      <c r="I12" s="4"/>
+      <c r="J12" s="4"/>
+      <c r="K12" s="4"/>
+      <c r="L12" s="3"/>
+    </row>
+    <row r="13" spans="1:26">
+      <c r="A13" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
+      <c r="I13" s="4"/>
+      <c r="J13" s="4"/>
+      <c r="K13" s="4"/>
+      <c r="L13" s="3"/>
+    </row>
+    <row r="14" spans="1:26">
+      <c r="A14" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14" s="4"/>
+      <c r="H14" s="4"/>
+      <c r="I14" s="4"/>
+      <c r="J14" s="4"/>
+      <c r="K14" s="4"/>
+      <c r="L14" s="3"/>
+    </row>
+    <row r="15" spans="1:26">
+      <c r="A15" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G15" s="4"/>
+      <c r="H15" s="4"/>
+      <c r="I15" s="4"/>
+      <c r="J15" s="4"/>
+      <c r="K15" s="4"/>
+      <c r="L15" s="3"/>
+    </row>
+    <row r="16" spans="1:26">
+      <c r="A16" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G16" s="4"/>
+      <c r="H16" s="4"/>
+      <c r="I16" s="4"/>
+      <c r="J16" s="4"/>
+      <c r="K16" s="4"/>
+      <c r="L16" s="3"/>
+    </row>
+    <row r="17" spans="1:12">
+      <c r="A17" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G17" s="4"/>
+      <c r="H17" s="4"/>
+      <c r="I17" s="4"/>
+      <c r="J17" s="4"/>
+      <c r="K17" s="4"/>
+      <c r="L17" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1454,7 +1939,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z11"/>
+  <dimension ref="A1:Z17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" customWidth="1"/>
@@ -1464,7 +1949,7 @@
   <sheetData>
     <row r="1" spans="1:26" ht="25" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1545,19 +2030,19 @@
         <v>10</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -1568,22 +2053,22 @@
     </row>
     <row r="5" spans="1:26">
       <c r="A5" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -1594,22 +2079,22 @@
     </row>
     <row r="6" spans="1:26">
       <c r="A6" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>11</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -1620,22 +2105,22 @@
     </row>
     <row r="7" spans="1:26">
       <c r="A7" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -1646,22 +2131,22 @@
     </row>
     <row r="8" spans="1:26">
       <c r="A8" s="2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -1672,22 +2157,22 @@
     </row>
     <row r="9" spans="1:26">
       <c r="A9" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -1698,22 +2183,22 @@
     </row>
     <row r="10" spans="1:26">
       <c r="A10" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -1724,22 +2209,22 @@
     </row>
     <row r="11" spans="1:26">
       <c r="A11" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -1747,6 +2232,162 @@
       <c r="J11" s="4"/>
       <c r="K11" s="4"/>
       <c r="L11" s="3"/>
+    </row>
+    <row r="12" spans="1:26">
+      <c r="A12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" s="4"/>
+      <c r="H12" s="4"/>
+      <c r="I12" s="4"/>
+      <c r="J12" s="4"/>
+      <c r="K12" s="4"/>
+      <c r="L12" s="3"/>
+    </row>
+    <row r="13" spans="1:26">
+      <c r="A13" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
+      <c r="I13" s="4"/>
+      <c r="J13" s="4"/>
+      <c r="K13" s="4"/>
+      <c r="L13" s="3"/>
+    </row>
+    <row r="14" spans="1:26">
+      <c r="A14" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14" s="4"/>
+      <c r="H14" s="4"/>
+      <c r="I14" s="4"/>
+      <c r="J14" s="4"/>
+      <c r="K14" s="4"/>
+      <c r="L14" s="3"/>
+    </row>
+    <row r="15" spans="1:26">
+      <c r="A15" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G15" s="4"/>
+      <c r="H15" s="4"/>
+      <c r="I15" s="4"/>
+      <c r="J15" s="4"/>
+      <c r="K15" s="4"/>
+      <c r="L15" s="3"/>
+    </row>
+    <row r="16" spans="1:26">
+      <c r="A16" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G16" s="4"/>
+      <c r="H16" s="4"/>
+      <c r="I16" s="4"/>
+      <c r="J16" s="4"/>
+      <c r="K16" s="4"/>
+      <c r="L16" s="3"/>
+    </row>
+    <row r="17" spans="1:12">
+      <c r="A17" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G17" s="4"/>
+      <c r="H17" s="4"/>
+      <c r="I17" s="4"/>
+      <c r="J17" s="4"/>
+      <c r="K17" s="4"/>
+      <c r="L17" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1760,512 +2401,280 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z11"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" customWidth="1"/>
-    <col min="2" max="11" width="8.7109375" customWidth="1"/>
-    <col min="12" max="12" width="15.7109375" customWidth="1"/>
+    <col min="2" max="5" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="25" customHeight="1">
+    <row r="1" spans="1:5" ht="25" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
-      <c r="P1" s="1"/>
-      <c r="Q1" s="1"/>
-      <c r="R1" s="1"/>
-      <c r="S1" s="1"/>
-      <c r="T1" s="1"/>
-      <c r="U1" s="1"/>
-      <c r="V1" s="1"/>
-      <c r="W1" s="1"/>
-      <c r="X1" s="1"/>
-      <c r="Y1" s="1"/>
-      <c r="Z1" s="1"/>
-    </row>
-    <row r="2" spans="1:26" ht="20" customHeight="1">
+    </row>
+    <row r="2" spans="1:5" ht="20" customHeight="1">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:26" ht="20" customHeight="1">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L3" s="1"/>
-    </row>
-    <row r="4" spans="1:26">
-      <c r="A4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
-      <c r="L4" s="3"/>
-    </row>
-    <row r="5" spans="1:26">
-      <c r="A5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="4"/>
-      <c r="L5" s="3"/>
-    </row>
-    <row r="6" spans="1:26">
-      <c r="A6" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
-      <c r="I6" s="4"/>
-      <c r="J6" s="4"/>
-      <c r="K6" s="4"/>
-      <c r="L6" s="3"/>
-    </row>
-    <row r="7" spans="1:26">
-      <c r="A7" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
-      <c r="L7" s="3"/>
-    </row>
-    <row r="8" spans="1:26">
-      <c r="A8" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
-      <c r="I8" s="4"/>
-      <c r="J8" s="4"/>
-      <c r="K8" s="4"/>
-      <c r="L8" s="3"/>
-    </row>
-    <row r="9" spans="1:26">
-      <c r="A9" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
-      <c r="I9" s="4"/>
-      <c r="J9" s="4"/>
-      <c r="K9" s="4"/>
-      <c r="L9" s="3"/>
-    </row>
-    <row r="10" spans="1:26">
-      <c r="A10" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
-      <c r="I10" s="4"/>
-      <c r="J10" s="4"/>
-      <c r="K10" s="4"/>
-      <c r="L10" s="3"/>
-    </row>
-    <row r="11" spans="1:26">
-      <c r="A11" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4"/>
-      <c r="I11" s="4"/>
-      <c r="J11" s="4"/>
-      <c r="K11" s="4"/>
-      <c r="L11" s="3"/>
-    </row>
-  </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A1:Z1"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="L2:L3"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="20.7109375" customWidth="1"/>
-    <col min="2" max="6" width="15.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" ht="25" customHeight="1">
-      <c r="A1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-    </row>
-    <row r="2" spans="1:6" ht="20" customHeight="1">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="D3" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
-      <c r="A4" s="2" t="s">
-        <v>12</v>
-      </c>
       <c r="B4" s="3" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="C4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="E6" s="3" t="s">
+      <c r="E8" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="F6" s="3" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
-      <c r="A7" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" s="3" t="s">
+      <c r="D9" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F7" s="3" t="s">
+      <c r="E9" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" s="3" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="8" spans="1:6">
-      <c r="A8" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
-      <c r="A9" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6">
-      <c r="A10" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="D10" s="3" t="s">
+      <c r="D11" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="E10" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>32</v>
+      <c r="C12" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix master_input and manual constraints
</commit_message>
<xml_diff>
--- a/DATA/schedule.xlsx
+++ b/DATA/schedule.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="42">
   <si>
     <t>Monday - [Insert Date]</t>
   </si>
@@ -50,58 +50,55 @@
     <t>Comments / Late</t>
   </si>
   <si>
-    <t>Chisholm Teddy</t>
+    <t>Akinsanmi, Fayo</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Chisholm, Teddy</t>
+  </si>
+  <si>
+    <t>Court 2</t>
   </si>
   <si>
     <t>Court 1</t>
   </si>
   <si>
-    <t>Court 2</t>
-  </si>
-  <si>
-    <t>Enkhjargal Manlai</t>
-  </si>
-  <si>
-    <t>-</t>
+    <t>Enkhjargal, Manlai</t>
   </si>
   <si>
     <t>Court 3</t>
   </si>
   <si>
-    <t>Gray Caroline</t>
-  </si>
-  <si>
-    <t>Huang Jason</t>
-  </si>
-  <si>
-    <t>Kerrigan Declan</t>
-  </si>
-  <si>
-    <t>Kevin Huang</t>
-  </si>
-  <si>
-    <t>Little Patrick</t>
-  </si>
-  <si>
-    <t>Nguyen Jinnie</t>
-  </si>
-  <si>
-    <t>Nguyen Millie</t>
-  </si>
-  <si>
-    <t>Pineo Kyle</t>
-  </si>
-  <si>
-    <t>Roix Aiden</t>
-  </si>
-  <si>
-    <t>Wasser David</t>
-  </si>
-  <si>
-    <t>Xu Ryan</t>
-  </si>
-  <si>
-    <t>Zaya Maria</t>
+    <t>Gray, Caroline</t>
+  </si>
+  <si>
+    <t>Huang, Jason</t>
+  </si>
+  <si>
+    <t>Kerrigan, Declan</t>
+  </si>
+  <si>
+    <t>Kevin, Huang</t>
+  </si>
+  <si>
+    <t>Little, Patrick</t>
+  </si>
+  <si>
+    <t>Pineo, Kyle</t>
+  </si>
+  <si>
+    <t>Roix, Aiden</t>
+  </si>
+  <si>
+    <t>Wasser, David</t>
+  </si>
+  <si>
+    <t>Xu, Ryan</t>
+  </si>
+  <si>
+    <t>Zaya, Maria</t>
   </si>
   <si>
     <t>Tuesday - [Insert Date]</t>
@@ -131,31 +128,22 @@
     <t>6:30, 7:30, 8:30, 9:30, 10:30</t>
   </si>
   <si>
-    <t>7:30, 8:30, 9:30, 10:30</t>
+    <t>6:30, 7:30</t>
+  </si>
+  <si>
+    <t>8:30, 9:30, 10:30</t>
+  </si>
+  <si>
+    <t>6:30, 7:30, 8:30, 9:30</t>
+  </si>
+  <si>
+    <t>9:30, 10:30</t>
   </si>
   <si>
     <t>6:30, 7:30, 8:30</t>
   </si>
   <si>
-    <t>6:30, 7:30, 8:30, 9:30</t>
-  </si>
-  <si>
-    <t>8:30, 9:30, 10:30</t>
-  </si>
-  <si>
-    <t>6:30, 8:30</t>
-  </si>
-  <si>
-    <t>9:30, 10:30</t>
-  </si>
-  <si>
-    <t>8:30, 9:30</t>
-  </si>
-  <si>
-    <t>6:30, 8:30, 9:30, 10:30</t>
-  </si>
-  <si>
-    <t>6:30, 7:30</t>
+    <t>7:30, 8:30, 9:30</t>
   </si>
 </sst>
 </file>
@@ -553,7 +541,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z17"/>
+  <dimension ref="A1:Z16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" customWidth="1"/>
@@ -653,7 +641,7 @@
         <v>11</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>11</v>
@@ -667,22 +655,22 @@
     </row>
     <row r="5" spans="1:26">
       <c r="A5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>15</v>
-      </c>
       <c r="E5" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -693,22 +681,22 @@
     </row>
     <row r="6" spans="1:26">
       <c r="A6" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -725,16 +713,16 @@
         <v>11</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -751,16 +739,16 @@
         <v>14</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -774,7 +762,7 @@
         <v>19</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>11</v>
@@ -783,10 +771,10 @@
         <v>11</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -809,7 +797,7 @@
         <v>14</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>11</v>
@@ -826,19 +814,19 @@
         <v>21</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -852,19 +840,19 @@
         <v>22</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -878,19 +866,19 @@
         <v>23</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -904,13 +892,13 @@
         <v>24</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>11</v>
@@ -930,19 +918,19 @@
         <v>25</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -965,7 +953,7 @@
         <v>11</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F16" s="3" t="s">
         <v>14</v>
@@ -976,32 +964,6 @@
       <c r="J16" s="4"/>
       <c r="K16" s="4"/>
       <c r="L16" s="3"/>
-    </row>
-    <row r="17" spans="1:12">
-      <c r="A17" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
-      <c r="I17" s="4"/>
-      <c r="J17" s="4"/>
-      <c r="K17" s="4"/>
-      <c r="L17" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1015,7 +977,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z17"/>
+  <dimension ref="A1:Z16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" customWidth="1"/>
@@ -1025,7 +987,7 @@
   <sheetData>
     <row r="1" spans="1:26" ht="25" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1106,19 +1068,19 @@
         <v>10</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -1129,22 +1091,22 @@
     </row>
     <row r="5" spans="1:26">
       <c r="A5" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -1155,7 +1117,7 @@
     </row>
     <row r="6" spans="1:26">
       <c r="A6" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>11</v>
@@ -1164,13 +1126,13 @@
         <v>11</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -1184,19 +1146,19 @@
         <v>17</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>14</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -1210,19 +1172,19 @@
         <v>18</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>11</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -1236,19 +1198,19 @@
         <v>19</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>14</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -1262,16 +1224,16 @@
         <v>20</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>11</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>11</v>
@@ -1288,19 +1250,19 @@
         <v>21</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -1314,19 +1276,19 @@
         <v>22</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -1340,19 +1302,19 @@
         <v>23</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -1366,10 +1328,10 @@
         <v>24</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>11</v>
@@ -1378,7 +1340,7 @@
         <v>11</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -1392,19 +1354,19 @@
         <v>25</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -1421,16 +1383,16 @@
         <v>11</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -1438,32 +1400,6 @@
       <c r="J16" s="4"/>
       <c r="K16" s="4"/>
       <c r="L16" s="3"/>
-    </row>
-    <row r="17" spans="1:12">
-      <c r="A17" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
-      <c r="I17" s="4"/>
-      <c r="J17" s="4"/>
-      <c r="K17" s="4"/>
-      <c r="L17" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1477,7 +1413,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z17"/>
+  <dimension ref="A1:Z16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" customWidth="1"/>
@@ -1487,7 +1423,7 @@
   <sheetData>
     <row r="1" spans="1:26" ht="25" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1568,19 +1504,19 @@
         <v>10</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -1591,22 +1527,22 @@
     </row>
     <row r="5" spans="1:26">
       <c r="A5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>12</v>
-      </c>
       <c r="C5" s="3" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>14</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -1617,22 +1553,22 @@
     </row>
     <row r="6" spans="1:26">
       <c r="A6" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -1649,13 +1585,13 @@
         <v>11</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>11</v>
@@ -1672,19 +1608,19 @@
         <v>18</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>11</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -1698,19 +1634,19 @@
         <v>19</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -1724,19 +1660,19 @@
         <v>20</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>14</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -1750,19 +1686,19 @@
         <v>21</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>11</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -1776,19 +1712,19 @@
         <v>22</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -1811,7 +1747,7 @@
         <v>14</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F13" s="3" t="s">
         <v>14</v>
@@ -1834,10 +1770,10 @@
         <v>14</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F14" s="3" t="s">
         <v>14</v>
@@ -1854,13 +1790,13 @@
         <v>25</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>11</v>
@@ -1880,19 +1816,19 @@
         <v>26</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -1900,32 +1836,6 @@
       <c r="J16" s="4"/>
       <c r="K16" s="4"/>
       <c r="L16" s="3"/>
-    </row>
-    <row r="17" spans="1:12">
-      <c r="A17" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
-      <c r="I17" s="4"/>
-      <c r="J17" s="4"/>
-      <c r="K17" s="4"/>
-      <c r="L17" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1939,7 +1849,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z17"/>
+  <dimension ref="A1:Z16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" customWidth="1"/>
@@ -1949,7 +1859,7 @@
   <sheetData>
     <row r="1" spans="1:26" ht="25" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2030,19 +1940,19 @@
         <v>10</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -2053,7 +1963,7 @@
     </row>
     <row r="5" spans="1:26">
       <c r="A5" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>11</v>
@@ -2062,13 +1972,13 @@
         <v>11</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -2079,22 +1989,22 @@
     </row>
     <row r="6" spans="1:26">
       <c r="A6" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>11</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -2108,19 +2018,19 @@
         <v>17</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -2134,19 +2044,19 @@
         <v>18</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -2166,13 +2076,13 @@
         <v>11</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -2186,19 +2096,19 @@
         <v>20</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G10" s="4"/>
       <c r="H10" s="4"/>
@@ -2212,7 +2122,7 @@
         <v>21</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>11</v>
@@ -2221,10 +2131,10 @@
         <v>11</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -2238,19 +2148,19 @@
         <v>22</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
@@ -2264,19 +2174,19 @@
         <v>23</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -2290,19 +2200,19 @@
         <v>24</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -2319,16 +2229,16 @@
         <v>14</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -2342,19 +2252,19 @@
         <v>26</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>11</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -2362,32 +2272,6 @@
       <c r="J16" s="4"/>
       <c r="K16" s="4"/>
       <c r="L16" s="3"/>
-    </row>
-    <row r="17" spans="1:12">
-      <c r="A17" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
-      <c r="I17" s="4"/>
-      <c r="J17" s="4"/>
-      <c r="K17" s="4"/>
-      <c r="L17" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2401,7 +2285,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" customWidth="1"/>
@@ -2410,7 +2294,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="25" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2422,16 +2306,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>34</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -2439,50 +2323,50 @@
         <v>10</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>36</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>37</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>38</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>38</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>38</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -2490,16 +2374,16 @@
         <v>17</v>
       </c>
       <c r="B6" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>14</v>
-      </c>
       <c r="D6" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>36</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -2507,16 +2391,16 @@
         <v>18</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>41</v>
+        <v>3</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -2524,16 +2408,16 @@
         <v>19</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>14</v>
+        <v>38</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>3</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>38</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -2541,16 +2425,16 @@
         <v>20</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>38</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -2558,16 +2442,16 @@
         <v>21</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>38</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -2575,16 +2459,16 @@
         <v>22</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -2592,16 +2476,16 @@
         <v>23</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -2609,16 +2493,16 @@
         <v>24</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>36</v>
+        <v>7</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -2626,16 +2510,16 @@
         <v>25</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -2643,33 +2527,16 @@
         <v>26</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5">
-      <c r="A16" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>38</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Look and feel changes
</commit_message>
<xml_diff>
--- a/DATA/schedule.xlsx
+++ b/DATA/schedule.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="45">
   <si>
     <t>Monday - [Insert Date]</t>
   </si>
@@ -59,16 +59,16 @@
     <t>Chisholm, Teddy</t>
   </si>
   <si>
-    <t>Court 2</t>
-  </si>
-  <si>
-    <t>Court 1</t>
-  </si>
-  <si>
     <t>Enkhjargal, Manlai</t>
   </si>
   <si>
-    <t>Court 3</t>
+    <t>3</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>2</t>
   </si>
   <si>
     <t>Gray, Caroline</t>
@@ -86,6 +86,12 @@
     <t>Little, Patrick</t>
   </si>
   <si>
+    <t>Nguyen, Jinnie</t>
+  </si>
+  <si>
+    <t>Nguyen, Millie</t>
+  </si>
+  <si>
     <t>Pineo, Kyle</t>
   </si>
   <si>
@@ -125,22 +131,25 @@
     <t>Thursday</t>
   </si>
   <si>
+    <t>6:30, 7:30</t>
+  </si>
+  <si>
+    <t>6:30, 7:30, 8:30</t>
+  </si>
+  <si>
     <t>6:30, 7:30, 8:30, 9:30, 10:30</t>
   </si>
   <si>
-    <t>6:30, 7:30</t>
+    <t>6:30, 7:30, 8:30, 9:30</t>
+  </si>
+  <si>
+    <t>8:30, 9:30</t>
   </si>
   <si>
     <t>8:30, 9:30, 10:30</t>
   </si>
   <si>
-    <t>6:30, 7:30, 8:30, 9:30</t>
-  </si>
-  <si>
     <t>9:30, 10:30</t>
-  </si>
-  <si>
-    <t>6:30, 7:30, 8:30</t>
   </si>
   <si>
     <t>7:30, 8:30, 9:30</t>
@@ -541,7 +550,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z16"/>
+  <dimension ref="A1:Z19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" customWidth="1"/>
@@ -655,7 +664,7 @@
     </row>
     <row r="5" spans="1:26">
       <c r="A5" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>11</v>
@@ -664,13 +673,13 @@
         <v>11</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -681,22 +690,22 @@
     </row>
     <row r="6" spans="1:26">
       <c r="A6" s="2" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -707,19 +716,19 @@
     </row>
     <row r="7" spans="1:26">
       <c r="A7" s="2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>11</v>
@@ -733,22 +742,22 @@
     </row>
     <row r="8" spans="1:26">
       <c r="A8" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
@@ -759,22 +768,22 @@
     </row>
     <row r="9" spans="1:26">
       <c r="A9" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>14</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -785,19 +794,19 @@
     </row>
     <row r="10" spans="1:26">
       <c r="A10" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>11</v>
@@ -811,16 +820,16 @@
     </row>
     <row r="11" spans="1:26">
       <c r="A11" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>11</v>
@@ -837,16 +846,16 @@
     </row>
     <row r="12" spans="1:26">
       <c r="A12" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>11</v>
@@ -863,7 +872,7 @@
     </row>
     <row r="13" spans="1:26">
       <c r="A13" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>11</v>
@@ -872,13 +881,13 @@
         <v>11</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -889,7 +898,7 @@
     </row>
     <row r="14" spans="1:26">
       <c r="A14" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>11</v>
@@ -898,13 +907,13 @@
         <v>11</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -915,19 +924,19 @@
     </row>
     <row r="15" spans="1:26">
       <c r="A15" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="F15" s="3" t="s">
         <v>11</v>
@@ -941,7 +950,7 @@
     </row>
     <row r="16" spans="1:26">
       <c r="A16" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>11</v>
@@ -953,10 +962,10 @@
         <v>11</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -964,6 +973,84 @@
       <c r="J16" s="4"/>
       <c r="K16" s="4"/>
       <c r="L16" s="3"/>
+    </row>
+    <row r="17" spans="1:12">
+      <c r="A17" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G17" s="4"/>
+      <c r="H17" s="4"/>
+      <c r="I17" s="4"/>
+      <c r="J17" s="4"/>
+      <c r="K17" s="4"/>
+      <c r="L17" s="3"/>
+    </row>
+    <row r="18" spans="1:12">
+      <c r="A18" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G18" s="4"/>
+      <c r="H18" s="4"/>
+      <c r="I18" s="4"/>
+      <c r="J18" s="4"/>
+      <c r="K18" s="4"/>
+      <c r="L18" s="3"/>
+    </row>
+    <row r="19" spans="1:12">
+      <c r="A19" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G19" s="4"/>
+      <c r="H19" s="4"/>
+      <c r="I19" s="4"/>
+      <c r="J19" s="4"/>
+      <c r="K19" s="4"/>
+      <c r="L19" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -977,7 +1064,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z16"/>
+  <dimension ref="A1:Z19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" customWidth="1"/>
@@ -987,7 +1074,7 @@
   <sheetData>
     <row r="1" spans="1:26" ht="25" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1068,19 +1155,19 @@
         <v>10</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>14</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -1091,13 +1178,13 @@
     </row>
     <row r="5" spans="1:26">
       <c r="A5" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>11</v>
@@ -1117,7 +1204,7 @@
     </row>
     <row r="6" spans="1:26">
       <c r="A6" s="2" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>11</v>
@@ -1143,19 +1230,19 @@
     </row>
     <row r="7" spans="1:26">
       <c r="A7" s="2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>11</v>
@@ -1169,16 +1256,16 @@
     </row>
     <row r="8" spans="1:26">
       <c r="A8" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>11</v>
@@ -1195,19 +1282,19 @@
     </row>
     <row r="9" spans="1:26">
       <c r="A9" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>11</v>
@@ -1221,19 +1308,19 @@
     </row>
     <row r="10" spans="1:26">
       <c r="A10" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>11</v>
@@ -1247,22 +1334,22 @@
     </row>
     <row r="11" spans="1:26">
       <c r="A11" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
@@ -1273,7 +1360,7 @@
     </row>
     <row r="12" spans="1:26">
       <c r="A12" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>11</v>
@@ -1282,10 +1369,10 @@
         <v>11</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="F12" s="3" t="s">
         <v>11</v>
@@ -1299,10 +1386,10 @@
     </row>
     <row r="13" spans="1:26">
       <c r="A13" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>11</v>
@@ -1325,7 +1412,7 @@
     </row>
     <row r="14" spans="1:26">
       <c r="A14" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>11</v>
@@ -1340,7 +1427,7 @@
         <v>11</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -1351,22 +1438,22 @@
     </row>
     <row r="15" spans="1:26">
       <c r="A15" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
@@ -1377,22 +1464,22 @@
     </row>
     <row r="16" spans="1:26">
       <c r="A16" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
@@ -1400,6 +1487,84 @@
       <c r="J16" s="4"/>
       <c r="K16" s="4"/>
       <c r="L16" s="3"/>
+    </row>
+    <row r="17" spans="1:12">
+      <c r="A17" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G17" s="4"/>
+      <c r="H17" s="4"/>
+      <c r="I17" s="4"/>
+      <c r="J17" s="4"/>
+      <c r="K17" s="4"/>
+      <c r="L17" s="3"/>
+    </row>
+    <row r="18" spans="1:12">
+      <c r="A18" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G18" s="4"/>
+      <c r="H18" s="4"/>
+      <c r="I18" s="4"/>
+      <c r="J18" s="4"/>
+      <c r="K18" s="4"/>
+      <c r="L18" s="3"/>
+    </row>
+    <row r="19" spans="1:12">
+      <c r="A19" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G19" s="4"/>
+      <c r="H19" s="4"/>
+      <c r="I19" s="4"/>
+      <c r="J19" s="4"/>
+      <c r="K19" s="4"/>
+      <c r="L19" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1413,7 +1578,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z16"/>
+  <dimension ref="A1:Z19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" customWidth="1"/>
@@ -1423,7 +1588,7 @@
   <sheetData>
     <row r="1" spans="1:26" ht="25" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1527,19 +1692,19 @@
     </row>
     <row r="5" spans="1:26">
       <c r="A5" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>11</v>
@@ -1553,22 +1718,22 @@
     </row>
     <row r="6" spans="1:26">
       <c r="A6" s="2" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -1579,10 +1744,10 @@
     </row>
     <row r="7" spans="1:26">
       <c r="A7" s="2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>11</v>
@@ -1605,10 +1770,10 @@
     </row>
     <row r="8" spans="1:26">
       <c r="A8" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>11</v>
@@ -1631,10 +1796,10 @@
     </row>
     <row r="9" spans="1:26">
       <c r="A9" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>11</v>
@@ -1657,19 +1822,19 @@
     </row>
     <row r="10" spans="1:26">
       <c r="A10" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F10" s="3" t="s">
         <v>11</v>
@@ -1683,16 +1848,16 @@
     </row>
     <row r="11" spans="1:26">
       <c r="A11" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>11</v>
@@ -1709,16 +1874,16 @@
     </row>
     <row r="12" spans="1:26">
       <c r="A12" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>11</v>
@@ -1735,7 +1900,7 @@
     </row>
     <row r="13" spans="1:26">
       <c r="A13" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>11</v>
@@ -1744,13 +1909,13 @@
         <v>11</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
@@ -1761,22 +1926,22 @@
     </row>
     <row r="14" spans="1:26">
       <c r="A14" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
@@ -1787,7 +1952,7 @@
     </row>
     <row r="15" spans="1:26">
       <c r="A15" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>11</v>
@@ -1813,7 +1978,7 @@
     </row>
     <row r="16" spans="1:26">
       <c r="A16" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>11</v>
@@ -1836,6 +2001,84 @@
       <c r="J16" s="4"/>
       <c r="K16" s="4"/>
       <c r="L16" s="3"/>
+    </row>
+    <row r="17" spans="1:12">
+      <c r="A17" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G17" s="4"/>
+      <c r="H17" s="4"/>
+      <c r="I17" s="4"/>
+      <c r="J17" s="4"/>
+      <c r="K17" s="4"/>
+      <c r="L17" s="3"/>
+    </row>
+    <row r="18" spans="1:12">
+      <c r="A18" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G18" s="4"/>
+      <c r="H18" s="4"/>
+      <c r="I18" s="4"/>
+      <c r="J18" s="4"/>
+      <c r="K18" s="4"/>
+      <c r="L18" s="3"/>
+    </row>
+    <row r="19" spans="1:12">
+      <c r="A19" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G19" s="4"/>
+      <c r="H19" s="4"/>
+      <c r="I19" s="4"/>
+      <c r="J19" s="4"/>
+      <c r="K19" s="4"/>
+      <c r="L19" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -1849,7 +2092,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z16"/>
+  <dimension ref="A1:Z19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" customWidth="1"/>
@@ -1859,7 +2102,7 @@
   <sheetData>
     <row r="1" spans="1:26" ht="25" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1940,13 +2183,13 @@
         <v>10</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>11</v>
@@ -1963,16 +2206,16 @@
     </row>
     <row r="5" spans="1:26">
       <c r="A5" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>11</v>
@@ -1989,10 +2232,10 @@
     </row>
     <row r="6" spans="1:26">
       <c r="A6" s="2" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>11</v>
@@ -2015,13 +2258,13 @@
     </row>
     <row r="7" spans="1:26">
       <c r="A7" s="2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>11</v>
@@ -2041,16 +2284,16 @@
     </row>
     <row r="8" spans="1:26">
       <c r="A8" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>11</v>
@@ -2067,7 +2310,7 @@
     </row>
     <row r="9" spans="1:26">
       <c r="A9" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>11</v>
@@ -2093,7 +2336,7 @@
     </row>
     <row r="10" spans="1:26">
       <c r="A10" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>11</v>
@@ -2119,7 +2362,7 @@
     </row>
     <row r="11" spans="1:26">
       <c r="A11" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>11</v>
@@ -2145,7 +2388,7 @@
     </row>
     <row r="12" spans="1:26">
       <c r="A12" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>11</v>
@@ -2171,16 +2414,16 @@
     </row>
     <row r="13" spans="1:26">
       <c r="A13" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>11</v>
@@ -2197,7 +2440,7 @@
     </row>
     <row r="14" spans="1:26">
       <c r="A14" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>11</v>
@@ -2223,10 +2466,10 @@
     </row>
     <row r="15" spans="1:26">
       <c r="A15" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>11</v>
@@ -2249,7 +2492,7 @@
     </row>
     <row r="16" spans="1:26">
       <c r="A16" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>11</v>
@@ -2272,6 +2515,84 @@
       <c r="J16" s="4"/>
       <c r="K16" s="4"/>
       <c r="L16" s="3"/>
+    </row>
+    <row r="17" spans="1:12">
+      <c r="A17" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G17" s="4"/>
+      <c r="H17" s="4"/>
+      <c r="I17" s="4"/>
+      <c r="J17" s="4"/>
+      <c r="K17" s="4"/>
+      <c r="L17" s="3"/>
+    </row>
+    <row r="18" spans="1:12">
+      <c r="A18" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G18" s="4"/>
+      <c r="H18" s="4"/>
+      <c r="I18" s="4"/>
+      <c r="J18" s="4"/>
+      <c r="K18" s="4"/>
+      <c r="L18" s="3"/>
+    </row>
+    <row r="19" spans="1:12">
+      <c r="A19" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G19" s="4"/>
+      <c r="H19" s="4"/>
+      <c r="I19" s="4"/>
+      <c r="J19" s="4"/>
+      <c r="K19" s="4"/>
+      <c r="L19" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2285,7 +2606,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.7109375" customWidth="1"/>
@@ -2294,7 +2615,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="25" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2306,16 +2627,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -2326,13 +2647,13 @@
         <v>11</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>11</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -2340,13 +2661,13 @@
         <v>12</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>37</v>
+        <v>11</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>11</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>11</v>
@@ -2354,19 +2675,19 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>11</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -2383,7 +2704,7 @@
         <v>11</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -2391,13 +2712,13 @@
         <v>18</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>11</v>
@@ -2408,13 +2729,13 @@
         <v>19</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>11</v>
@@ -2425,7 +2746,7 @@
         <v>20</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>11</v>
@@ -2445,10 +2766,10 @@
         <v>11</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>5</v>
+        <v>38</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>11</v>
@@ -2459,16 +2780,16 @@
         <v>22</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>11</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>11</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -2476,13 +2797,13 @@
         <v>23</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>11</v>
@@ -2493,13 +2814,13 @@
         <v>24</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>35</v>
+        <v>11</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>11</v>
@@ -2513,13 +2834,13 @@
         <v>11</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>11</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -2527,15 +2848,49 @@
         <v>26</v>
       </c>
       <c r="B15" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C15" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>11</v>
-      </c>
       <c r="E15" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E17" s="3" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>